<commit_message>
schema redesign (org_id, natural keys, part_no refs) + real login (scrypt, user groups, JWT)
- drop warehouse_code/warehouse_sections/sub_inventories -> org_id (integer office)
- receiving_orders.ref_no -> batch_no; picking_orders.ref_no -> order_no (UNIQUE, sync key)
- receiving_invoice_items.qty -> line_qty, box_id -> ctn_no; parts referenced by part_no
- external_id removed; ingest upserts key on batch_no/order_no
- box ids BOX-<kind>-<YYYYMMDD>-<seq> (no warehouse segment)
- auth: scrypt password hashing (lazy legacy upgrade), user_groups +
  user_group_members (many-to-many, replaces users.role), JWT bearer enforced
  on all routes except /health, /auth/login, /dev/*; actorId from token
- web/admin clients send bearer token; SSE via ?token=; admin user-groups CRUD
- put-away scan-box feature; shelf_boxes order derived from items
- migrations 0014 + 0015; backend 98 tests, web 178 tests green
</commit_message>
<xml_diff>
--- a/new_seed/subInventories.xlsx
+++ b/new_seed/subInventories.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\work\docpal\warehouse-pda\new_seed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04B7647B-A459-4948-8A3F-7BE97DCEBB1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD3A21CB-E4D5-4ADE-92D8-166E3819A6A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{0A45231D-5C08-43FC-9205-77E8B8F5E855}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{0A45231D-5C08-43FC-9205-77E8B8F5E855}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="28">
   <si>
     <t>warehouseSections</t>
   </si>
@@ -120,6 +120,9 @@
   </si>
   <si>
     <t>HUAWEI-CAR</t>
+  </si>
+  <si>
+    <t>DEFAULT</t>
   </si>
 </sst>
 </file>
@@ -170,11 +173,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -509,15 +511,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{179B4C2D-3A50-4F7A-88FA-8F0F76756055}">
-  <dimension ref="A1:D20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5703125" customWidth="1"/>
     <col min="2" max="2" width="22.42578125" customWidth="1"/>
     <col min="3" max="4" width="22.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -529,7 +531,7 @@
       </c>
       <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -541,7 +543,7 @@
       </c>
       <c r="D2" s="2"/>
     </row>
-    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -553,7 +555,7 @@
       </c>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -565,7 +567,7 @@
       </c>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -577,7 +579,7 @@
       </c>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -589,7 +591,7 @@
       </c>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
@@ -601,7 +603,7 @@
       </c>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
@@ -613,7 +615,7 @@
       </c>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
@@ -625,7 +627,7 @@
       </c>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
@@ -637,7 +639,7 @@
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>3</v>
       </c>
@@ -649,19 +651,19 @@
       </c>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="3"/>
-    </row>
-    <row r="13" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="D12" s="1"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>3</v>
       </c>
@@ -673,7 +675,7 @@
       </c>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>3</v>
       </c>
@@ -685,7 +687,7 @@
       </c>
       <c r="D14" s="2"/>
     </row>
-    <row r="15" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>3</v>
       </c>
@@ -697,19 +699,19 @@
       </c>
       <c r="D15" s="2"/>
     </row>
-    <row r="16" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D16" s="2"/>
     </row>
-    <row r="17" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>3</v>
       </c>
@@ -717,11 +719,11 @@
         <v>20</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D17" s="2"/>
     </row>
-    <row r="18" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>3</v>
       </c>
@@ -729,11 +731,11 @@
         <v>20</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D18" s="2"/>
     </row>
-    <row r="19" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>3</v>
       </c>
@@ -741,11 +743,11 @@
         <v>20</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D19" s="2"/>
     </row>
-    <row r="20" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>3</v>
       </c>
@@ -753,9 +755,32 @@
         <v>20</v>
       </c>
       <c r="C20" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D20" s="2"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D20" s="2"/>
+      <c r="D21" s="2"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>27</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>